<commit_message>
Sync supplementary materials with current submission package
</commit_message>
<xml_diff>
--- a/supplementary-material/Supplementary Table S10.xlsx
+++ b/supplementary-material/Supplementary Table S10.xlsx
@@ -4,9 +4,7 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/huhuiling/AI_Employment/4 paper：VR WCE/Supplement827/"/>
-    </mc:Choice>
+    <mc:Choice Requires="x15"/>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF22CB17-A1F4-DB47-9AE4-35CD4ED27452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>